<commit_message>
added histidine and more buffers
</commit_message>
<xml_diff>
--- a/reports/buffer_vs_water.xlsx
+++ b/reports/buffer_vs_water.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,92 +489,313 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MEA</t>
+          <t>BV</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>5.5</v>
       </c>
       <c r="C6" t="n">
-        <v>50</v>
+        <v>415</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MEA</t>
+          <t>BV</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>88</v>
+        <v>483</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MEA</t>
+          <t>BV</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5.5</v>
+        <v>6.5</v>
       </c>
       <c r="C8" t="n">
-        <v>116</v>
+        <v>537</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TPS</t>
+          <t>HIST</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>3.5</v>
       </c>
       <c r="C9" t="n">
-        <v>153</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TPS</t>
+          <t>HIST</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>4</v>
       </c>
       <c r="C10" t="n">
-        <v>194</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TPS</t>
+          <t>HIST</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>4.5</v>
       </c>
       <c r="C11" t="n">
-        <v>236</v>
+        <v>104</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TPS</t>
+          <t>HIST</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>5</v>
       </c>
       <c r="C12" t="n">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>HIST</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="C13" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>HIST</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>6</v>
+      </c>
+      <c r="C14" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>HIST</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="C15" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>MEA</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="C16" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>MEA</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>MEA</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C18" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>MEA</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>MEA</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="C20" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>MEA</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>6</v>
+      </c>
+      <c r="C21" t="n">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>MEA</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="C22" t="n">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="C23" t="n">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>4</v>
+      </c>
+      <c r="C24" t="n">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C25" t="n">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>5</v>
+      </c>
+      <c r="C26" t="n">
         <v>289</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="C27" t="n">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>6</v>
+      </c>
+      <c r="C28" t="n">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="C29" t="n">
+        <v>434</v>
       </c>
     </row>
   </sheetData>
@@ -588,7 +809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -604,10 +825,15 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>HIST</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>MEA</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>TPS</t>
         </is>
@@ -620,8 +846,13 @@
       <c r="B2" t="n">
         <v>221</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="n">
+        <v>60</v>
+      </c>
       <c r="D2" t="n">
+        <v>38</v>
+      </c>
+      <c r="E2" t="n">
         <v>153</v>
       </c>
     </row>
@@ -633,9 +864,12 @@
         <v>265</v>
       </c>
       <c r="C3" t="n">
+        <v>76</v>
+      </c>
+      <c r="D3" t="n">
         <v>50</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>194</v>
       </c>
     </row>
@@ -646,8 +880,13 @@
       <c r="B4" t="n">
         <v>303</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="n">
+        <v>104</v>
+      </c>
       <c r="D4" t="n">
+        <v>72</v>
+      </c>
+      <c r="E4" t="n">
         <v>236</v>
       </c>
     </row>
@@ -659,9 +898,12 @@
         <v>335</v>
       </c>
       <c r="C5" t="n">
+        <v>134</v>
+      </c>
+      <c r="D5" t="n">
         <v>88</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>289</v>
       </c>
     </row>
@@ -669,11 +911,52 @@
       <c r="A6" t="n">
         <v>5.5</v>
       </c>
-      <c r="B6" t="inlineStr"/>
+      <c r="B6" t="n">
+        <v>415</v>
+      </c>
       <c r="C6" t="n">
+        <v>163</v>
+      </c>
+      <c r="D6" t="n">
         <v>116</v>
       </c>
-      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="n">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>483</v>
+      </c>
+      <c r="C7" t="n">
+        <v>185</v>
+      </c>
+      <c r="D7" t="n">
+        <v>143</v>
+      </c>
+      <c r="E7" t="n">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="B8" t="n">
+        <v>537</v>
+      </c>
+      <c r="C8" t="n">
+        <v>228</v>
+      </c>
+      <c r="D8" t="n">
+        <v>171</v>
+      </c>
+      <c r="E8" t="n">
+        <v>434</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>